<commit_message>
Update India FGI — 2026-07-30
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Core" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Extended" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -77,7 +74,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -85,19 +82,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -105,7 +96,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1479"/>
+  <dimension ref="A1:H1481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -539,7 +530,7 @@
         <v>23.10756972111554</v>
       </c>
       <c r="D2" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E2" t="n">
         <v>35.45816733067729</v>
@@ -569,7 +560,7 @@
         <v>19.92031872509961</v>
       </c>
       <c r="D3" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E3" t="n">
         <v>49.00398406374502</v>
@@ -632,7 +623,7 @@
         <v>52.19123505976096</v>
       </c>
       <c r="E5" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="F5" t="n">
         <v>98.80478087649402</v>
@@ -659,7 +650,7 @@
         <v>17.92828685258964</v>
       </c>
       <c r="D6" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E6" t="n">
         <v>31.07569721115538</v>
@@ -683,7 +674,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="C7" t="n">
         <v>20.7171314741036</v>
@@ -719,7 +710,7 @@
         <v>22.70916334661355</v>
       </c>
       <c r="D8" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E8" t="n">
         <v>89.24302788844621</v>
@@ -749,7 +740,7 @@
         <v>27.09163346613546</v>
       </c>
       <c r="D9" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E9" t="n">
         <v>97.60956175298804</v>
@@ -779,7 +770,7 @@
         <v>26.69322709163346</v>
       </c>
       <c r="D10" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E10" t="n">
         <v>82.07171314741036</v>
@@ -809,7 +800,7 @@
         <v>25.4980079681275</v>
       </c>
       <c r="D11" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E11" t="n">
         <v>67.72908366533864</v>
@@ -926,7 +917,7 @@
         <v>54.58167330677291</v>
       </c>
       <c r="C15" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D15" t="n">
         <v>25.89641434262948</v>
@@ -1256,7 +1247,7 @@
         <v>92.82868525896414</v>
       </c>
       <c r="C26" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="D26" t="n">
         <v>51.79282868525896</v>
@@ -1316,7 +1307,7 @@
         <v>100</v>
       </c>
       <c r="C28" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="D28" t="n">
         <v>50.99601593625498</v>
@@ -1376,7 +1367,7 @@
         <v>100</v>
       </c>
       <c r="C30" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="D30" t="n">
         <v>50.59760956175299</v>
@@ -1526,7 +1517,7 @@
         <v>97.60956175298804</v>
       </c>
       <c r="C35" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="D35" t="n">
         <v>49.40239043824701</v>
@@ -2588,7 +2579,7 @@
         <v>50.99601593625498</v>
       </c>
       <c r="G70" t="n">
-        <v>54.10358565737051</v>
+        <v>54.10358565737052</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
@@ -2798,7 +2789,7 @@
         <v>23.50597609561753</v>
       </c>
       <c r="G77" t="n">
-        <v>52.90836653386454</v>
+        <v>52.90836653386455</v>
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
@@ -2825,7 +2816,7 @@
         <v>43.82470119521912</v>
       </c>
       <c r="F78" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G78" t="n">
         <v>48.84462151394423</v>
@@ -3218,7 +3209,7 @@
         <v>56.17529880478087</v>
       </c>
       <c r="G91" t="n">
-        <v>56.25498007968127</v>
+        <v>56.25498007968128</v>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
@@ -3368,7 +3359,7 @@
         <v>76.09561752988047</v>
       </c>
       <c r="G96" t="n">
-        <v>48.28685258964143</v>
+        <v>48.28685258964144</v>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
@@ -3545,7 +3536,7 @@
         <v>46.21513944223107</v>
       </c>
       <c r="F102" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="G102" t="n">
         <v>47.64940239043825</v>
@@ -3926,7 +3917,7 @@
         <v>98.80478087649402</v>
       </c>
       <c r="C115" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="D115" t="n">
         <v>38.64541832669322</v>
@@ -4676,7 +4667,7 @@
         <v>100</v>
       </c>
       <c r="C140" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="D140" t="n">
         <v>37.05179282868526</v>
@@ -4739,7 +4730,7 @@
         <v>69.32270916334662</v>
       </c>
       <c r="D142" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="E142" t="n">
         <v>90.83665338645416</v>
@@ -4769,7 +4760,7 @@
         <v>65.33864541832669</v>
       </c>
       <c r="D143" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="E143" t="n">
         <v>83.66533864541833</v>
@@ -5096,7 +5087,7 @@
         <v>98.40637450199203</v>
       </c>
       <c r="C154" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="D154" t="n">
         <v>34.66135458167331</v>
@@ -5132,7 +5123,7 @@
         <v>34.66135458167331</v>
       </c>
       <c r="E155" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F155" t="n">
         <v>68.52589641434263</v>
@@ -5786,7 +5777,7 @@
         <v>70.11952191235061</v>
       </c>
       <c r="C177" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D177" t="n">
         <v>12.35059760956175</v>
@@ -5855,7 +5846,7 @@
         <v>83.26693227091634</v>
       </c>
       <c r="F179" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="G179" t="n">
         <v>56.01593625498008</v>
@@ -5918,7 +5909,7 @@
         <v>33.46613545816733</v>
       </c>
       <c r="G181" t="n">
-        <v>52.43027888446215</v>
+        <v>52.43027888446216</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
@@ -6368,7 +6359,7 @@
         <v>8.764940239043826</v>
       </c>
       <c r="G196" t="n">
-        <v>28.28685258964143</v>
+        <v>28.28685258964144</v>
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
@@ -6389,7 +6380,7 @@
         <v>79.68127490039841</v>
       </c>
       <c r="D197" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E197" t="n">
         <v>49.00398406374502</v>
@@ -6608,7 +6599,7 @@
         <v>7.569721115537849</v>
       </c>
       <c r="G204" t="n">
-        <v>46.45418326693227</v>
+        <v>46.45418326693228</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
@@ -6623,7 +6614,7 @@
         </is>
       </c>
       <c r="B205" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C205" t="n">
         <v>48.60557768924303</v>
@@ -6689,7 +6680,7 @@
         <v>68.92430278884461</v>
       </c>
       <c r="D207" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E207" t="n">
         <v>44.22310756972112</v>
@@ -6929,7 +6920,7 @@
         <v>50.99601593625498</v>
       </c>
       <c r="D215" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="E215" t="n">
         <v>77.29083665338645</v>
@@ -6959,7 +6950,7 @@
         <v>40.63745019920319</v>
       </c>
       <c r="D216" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="E216" t="n">
         <v>69.7211155378486</v>
@@ -7145,7 +7136,7 @@
         <v>95.2191235059761</v>
       </c>
       <c r="F222" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G222" t="n">
         <v>49.48207171314742</v>
@@ -7223,7 +7214,7 @@
         </is>
       </c>
       <c r="B225" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C225" t="n">
         <v>91.23505976095618</v>
@@ -7793,7 +7784,7 @@
         </is>
       </c>
       <c r="B244" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="C244" t="n">
         <v>98.40637450199203</v>
@@ -7922,7 +7913,7 @@
         <v>14.34262948207172</v>
       </c>
       <c r="E248" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="F248" t="n">
         <v>45.81673306772908</v>
@@ -7943,7 +7934,7 @@
         </is>
       </c>
       <c r="B249" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C249" t="n">
         <v>95.61752988047807</v>
@@ -8315,7 +8306,7 @@
         <v>25.0996015936255</v>
       </c>
       <c r="F261" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="G261" t="n">
         <v>33.30677290836653</v>
@@ -8465,7 +8456,7 @@
         <v>12.35059760956175</v>
       </c>
       <c r="F266" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="G266" t="n">
         <v>30.199203187251</v>
@@ -8498,7 +8489,7 @@
         <v>16.33466135458167</v>
       </c>
       <c r="G267" t="n">
-        <v>26.37450199203187</v>
+        <v>26.37450199203188</v>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
@@ -8528,7 +8519,7 @@
         <v>33.06772908366533</v>
       </c>
       <c r="G268" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
@@ -8582,10 +8573,10 @@
         <v>11.95219123505976</v>
       </c>
       <c r="E270" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="F270" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G270" t="n">
         <v>33.38645418326693</v>
@@ -8645,7 +8636,7 @@
         <v>16.33466135458167</v>
       </c>
       <c r="F272" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G272" t="n">
         <v>29.8804780876494</v>
@@ -10142,7 +10133,7 @@
         <v>10.75697211155378</v>
       </c>
       <c r="E322" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F322" t="n">
         <v>43.42629482071713</v>
@@ -10358,7 +10349,7 @@
         <v>66.53386454183267</v>
       </c>
       <c r="G329" t="n">
-        <v>48.60557768924303</v>
+        <v>48.60557768924304</v>
       </c>
       <c r="H329" s="3" t="inlineStr">
         <is>
@@ -11252,7 +11243,7 @@
         <v>1.195219123505976</v>
       </c>
       <c r="E359" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="F359" t="n">
         <v>2.390438247011952</v>
@@ -11336,7 +11327,7 @@
         <v>7.569721115537849</v>
       </c>
       <c r="C362" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="D362" t="n">
         <v>1.593625498007968</v>
@@ -11705,7 +11696,7 @@
         <v>33.86454183266932</v>
       </c>
       <c r="F374" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G374" t="n">
         <v>28.68525896414343</v>
@@ -12158,7 +12149,7 @@
         <v>99.601593625498</v>
       </c>
       <c r="G389" t="n">
-        <v>60.63745019920319</v>
+        <v>60.6374501992032</v>
       </c>
       <c r="H389" s="4" t="inlineStr">
         <is>
@@ -12665,7 +12656,7 @@
         <v>61.75298804780876</v>
       </c>
       <c r="F406" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="G406" t="n">
         <v>25.65737051792829</v>
@@ -12812,7 +12803,7 @@
         <v>4.382470119521913</v>
       </c>
       <c r="E411" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="F411" t="n">
         <v>18.32669322709163</v>
@@ -13295,7 +13286,7 @@
         <v>94.42231075697212</v>
       </c>
       <c r="F427" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G427" t="n">
         <v>30.35856573705179</v>
@@ -13316,7 +13307,7 @@
         <v>3.98406374501992</v>
       </c>
       <c r="C428" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="D428" t="n">
         <v>25.0996015936255</v>
@@ -13679,7 +13670,7 @@
         <v>39.04382470119522</v>
       </c>
       <c r="D440" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E440" t="n">
         <v>86.85258964143426</v>
@@ -13853,7 +13844,7 @@
         </is>
       </c>
       <c r="B446" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C446" t="n">
         <v>39.04382470119522</v>
@@ -14129,7 +14120,7 @@
         <v>29.08366533864542</v>
       </c>
       <c r="D455" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E455" t="n">
         <v>39.04382470119522</v>
@@ -14702,7 +14693,7 @@
         <v>0</v>
       </c>
       <c r="E474" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="F474" t="n">
         <v>3.585657370517929</v>
@@ -14795,7 +14786,7 @@
         <v>92.43027888446214</v>
       </c>
       <c r="F477" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G477" t="n">
         <v>38.08764940239043</v>
@@ -15416,7 +15407,7 @@
         <v>8.764940239043826</v>
       </c>
       <c r="C498" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D498" t="n">
         <v>36.65338645418327</v>
@@ -15476,7 +15467,7 @@
         <v>7.968127490039841</v>
       </c>
       <c r="C500" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D500" t="n">
         <v>0</v>
@@ -15635,7 +15626,7 @@
         <v>95.61752988047807</v>
       </c>
       <c r="F505" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G505" t="n">
         <v>43.18725099601594</v>
@@ -16028,7 +16019,7 @@
         <v>72.50996015936255</v>
       </c>
       <c r="G518" t="n">
-        <v>54.10358565737051</v>
+        <v>54.10358565737052</v>
       </c>
       <c r="H518" s="3" t="inlineStr">
         <is>
@@ -17045,7 +17036,7 @@
         <v>42.23107569721115</v>
       </c>
       <c r="F552" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="G552" t="n">
         <v>49.9601593625498</v>
@@ -17108,7 +17099,7 @@
         <v>33.46613545816733</v>
       </c>
       <c r="G554" t="n">
-        <v>40.63745019920319</v>
+        <v>40.6374501992032</v>
       </c>
       <c r="H554" s="2" t="inlineStr">
         <is>
@@ -17216,7 +17207,7 @@
         <v>59.76095617529881</v>
       </c>
       <c r="C558" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D558" t="n">
         <v>16.73306772908366</v>
@@ -17255,10 +17246,10 @@
         <v>4.382470119521913</v>
       </c>
       <c r="F559" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G559" t="n">
-        <v>24.46215139442231</v>
+        <v>24.46215139442232</v>
       </c>
       <c r="H559" s="6" t="inlineStr">
         <is>
@@ -17555,7 +17546,7 @@
         <v>10.35856573705179</v>
       </c>
       <c r="F569" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G569" t="n">
         <v>27.96812749003984</v>
@@ -17582,10 +17573,10 @@
         <v>40.63745019920319</v>
       </c>
       <c r="E570" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F570" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G570" t="n">
         <v>39.52191235059761</v>
@@ -18332,7 +18323,7 @@
         <v>19.12350597609562</v>
       </c>
       <c r="E595" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="F595" t="n">
         <v>70.11952191235061</v>
@@ -18368,7 +18359,7 @@
         <v>67.33067729083665</v>
       </c>
       <c r="G596" t="n">
-        <v>57.92828685258963</v>
+        <v>57.92828685258964</v>
       </c>
       <c r="H596" s="4" t="inlineStr">
         <is>
@@ -18908,7 +18899,7 @@
         <v>42.23107569721115</v>
       </c>
       <c r="G614" t="n">
-        <v>56.73306772908366</v>
+        <v>56.73306772908367</v>
       </c>
       <c r="H614" s="4" t="inlineStr">
         <is>
@@ -19142,7 +19133,7 @@
         <v>16.73306772908366</v>
       </c>
       <c r="E622" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="F622" t="n">
         <v>19.12350597609562</v>
@@ -19205,7 +19196,7 @@
         <v>27.88844621513944</v>
       </c>
       <c r="F624" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G624" t="n">
         <v>43.42629482071713</v>
@@ -19265,7 +19256,7 @@
         <v>41.83266932270917</v>
       </c>
       <c r="F626" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G626" t="n">
         <v>52.50996015936255</v>
@@ -19355,7 +19346,7 @@
         <v>15.53784860557769</v>
       </c>
       <c r="F629" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="G629" t="n">
         <v>37.76892430278885</v>
@@ -19442,7 +19433,7 @@
         <v>16.73306772908366</v>
       </c>
       <c r="E632" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="F632" t="n">
         <v>15.1394422310757</v>
@@ -19775,7 +19766,7 @@
         <v>9.561752988047809</v>
       </c>
       <c r="F643" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G643" t="n">
         <v>27.72908366533865</v>
@@ -19862,7 +19853,7 @@
         <v>16.73306772908366</v>
       </c>
       <c r="E646" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="F646" t="n">
         <v>16.33466135458167</v>
@@ -19988,7 +19979,7 @@
         <v>25.89641434262948</v>
       </c>
       <c r="G650" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="H650" s="2" t="inlineStr">
         <is>
@@ -20282,7 +20273,7 @@
         <v>15.93625498007968</v>
       </c>
       <c r="E660" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F660" t="n">
         <v>35.85657370517929</v>
@@ -20558,7 +20549,7 @@
         <v>55.37848605577689</v>
       </c>
       <c r="G669" t="n">
-        <v>60.07968127490039</v>
+        <v>60.0796812749004</v>
       </c>
       <c r="H669" s="4" t="inlineStr">
         <is>
@@ -20633,7 +20624,7 @@
         </is>
       </c>
       <c r="B672" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C672" t="n">
         <v>92.82868525896414</v>
@@ -20882,7 +20873,7 @@
         <v>0</v>
       </c>
       <c r="E680" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F680" t="n">
         <v>10.35856573705179</v>
@@ -21005,7 +20996,7 @@
         <v>17.13147410358566</v>
       </c>
       <c r="F684" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="G684" t="n">
         <v>24.54183266932271</v>
@@ -21143,7 +21134,7 @@
         </is>
       </c>
       <c r="B689" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="C689" t="n">
         <v>100</v>
@@ -21398,7 +21389,7 @@
         <v>72.50996015936255</v>
       </c>
       <c r="G697" t="n">
-        <v>63.90438247011951</v>
+        <v>63.90438247011952</v>
       </c>
       <c r="H697" s="4" t="inlineStr">
         <is>
@@ -22589,7 +22580,7 @@
         <v>98.00796812749005</v>
       </c>
       <c r="D737" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="E737" t="n">
         <v>63.74501992031873</v>
@@ -23345,7 +23336,7 @@
         <v>15.1394422310757</v>
       </c>
       <c r="F762" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G762" t="n">
         <v>39.60159362549801</v>
@@ -23468,7 +23459,7 @@
         <v>19.12350597609562</v>
       </c>
       <c r="G766" t="n">
-        <v>44.46215139442231</v>
+        <v>44.46215139442232</v>
       </c>
       <c r="H766" s="2" t="inlineStr">
         <is>
@@ -23705,7 +23696,7 @@
         <v>28.68525896414343</v>
       </c>
       <c r="F774" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G774" t="n">
         <v>42.78884462151395</v>
@@ -24983,7 +24974,7 @@
         </is>
       </c>
       <c r="B817" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C817" t="n">
         <v>90.8366533864542</v>
@@ -26489,7 +26480,7 @@
         <v>17.52988047808765</v>
       </c>
       <c r="D867" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="E867" t="n">
         <v>37.45019920318725</v>
@@ -26525,7 +26516,7 @@
         <v>16.73306772908366</v>
       </c>
       <c r="F868" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="G868" t="n">
         <v>31.79282868525897</v>
@@ -26666,7 +26657,7 @@
         <v>88.84462151394422</v>
       </c>
       <c r="C873" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="D873" t="n">
         <v>26.29482071713147</v>
@@ -26912,10 +26903,10 @@
         <v>23.50597609561753</v>
       </c>
       <c r="E881" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="F881" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G881" t="n">
         <v>29.64143426294821</v>
@@ -26936,7 +26927,7 @@
         <v>79.2828685258964</v>
       </c>
       <c r="C882" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="D882" t="n">
         <v>25.89641434262948</v>
@@ -27086,7 +27077,7 @@
         <v>88.44621513944223</v>
       </c>
       <c r="C887" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="D887" t="n">
         <v>24.70119521912351</v>
@@ -27119,7 +27110,7 @@
         <v>9.561752988047814</v>
       </c>
       <c r="D888" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E888" t="n">
         <v>62.15139442231076</v>
@@ -27149,7 +27140,7 @@
         <v>11.95219123505976</v>
       </c>
       <c r="D889" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E889" t="n">
         <v>54.18326693227091</v>
@@ -27179,7 +27170,7 @@
         <v>5.976095617529879</v>
       </c>
       <c r="D890" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E890" t="n">
         <v>30.2788844621514</v>
@@ -27209,7 +27200,7 @@
         <v>5.179282868525888</v>
       </c>
       <c r="D891" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E891" t="n">
         <v>39.44223107569721</v>
@@ -27272,13 +27263,13 @@
         <v>24.70119521912351</v>
       </c>
       <c r="E893" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="F893" t="n">
         <v>52.58964143426294</v>
       </c>
       <c r="G893" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="H893" s="2" t="inlineStr">
         <is>
@@ -27299,7 +27290,7 @@
         <v>10.35856573705179</v>
       </c>
       <c r="D894" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="E894" t="n">
         <v>44.6215139442231</v>
@@ -27389,7 +27380,7 @@
         <v>19.12350597609563</v>
       </c>
       <c r="D897" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="E897" t="n">
         <v>47.80876494023904</v>
@@ -27446,7 +27437,7 @@
         <v>85.2589641434263</v>
       </c>
       <c r="C899" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D899" t="n">
         <v>22.31075697211155</v>
@@ -27518,7 +27509,7 @@
         <v>43.82470119521912</v>
       </c>
       <c r="G901" t="n">
-        <v>25.1792828685259</v>
+        <v>25.17928286852589</v>
       </c>
       <c r="H901" s="2" t="inlineStr">
         <is>
@@ -27608,7 +27599,7 @@
         <v>35.0597609561753</v>
       </c>
       <c r="G904" t="n">
-        <v>26.53386454183267</v>
+        <v>26.53386454183268</v>
       </c>
       <c r="H904" s="2" t="inlineStr">
         <is>
@@ -27785,7 +27776,7 @@
         <v>33.86454183266932</v>
       </c>
       <c r="F910" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="G910" t="n">
         <v>35.61752988047809</v>
@@ -27818,7 +27809,7 @@
         <v>37.84860557768924</v>
       </c>
       <c r="G911" t="n">
-        <v>46.45418326693227</v>
+        <v>46.45418326693228</v>
       </c>
       <c r="H911" s="3" t="inlineStr">
         <is>
@@ -27899,7 +27890,7 @@
         <v>70.91633466135458</v>
       </c>
       <c r="D914" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E914" t="n">
         <v>52.19123505976096</v>
@@ -28118,7 +28109,7 @@
         <v>56.17529880478087</v>
       </c>
       <c r="G921" t="n">
-        <v>29.24302788844622</v>
+        <v>29.24302788844621</v>
       </c>
       <c r="H921" s="2" t="inlineStr">
         <is>
@@ -28232,7 +28223,7 @@
         <v>19.52191235059761</v>
       </c>
       <c r="E925" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="F925" t="n">
         <v>77.68924302788844</v>
@@ -28358,7 +28349,7 @@
         <v>64.14342629482071</v>
       </c>
       <c r="G929" t="n">
-        <v>48.28685258964143</v>
+        <v>48.28685258964144</v>
       </c>
       <c r="H929" s="3" t="inlineStr">
         <is>
@@ -28673,7 +28664,7 @@
         </is>
       </c>
       <c r="B940" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="C940" t="n">
         <v>0.3984063745019881</v>
@@ -28748,7 +28739,7 @@
         <v>35.0597609561753</v>
       </c>
       <c r="G942" t="n">
-        <v>30.43824701195219</v>
+        <v>30.4382470119522</v>
       </c>
       <c r="H942" s="2" t="inlineStr">
         <is>
@@ -28898,7 +28889,7 @@
         <v>43.82470119521912</v>
       </c>
       <c r="G947" t="n">
-        <v>36.73306772908366</v>
+        <v>36.73306772908367</v>
       </c>
       <c r="H947" s="2" t="inlineStr">
         <is>
@@ -28928,7 +28919,7 @@
         <v>33.06772908366533</v>
       </c>
       <c r="G948" t="n">
-        <v>31.15537848605578</v>
+        <v>31.15537848605577</v>
       </c>
       <c r="H948" s="2" t="inlineStr">
         <is>
@@ -28979,7 +28970,7 @@
         <v>0.3984063745019881</v>
       </c>
       <c r="D950" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E950" t="n">
         <v>17.52988047808765</v>
@@ -29039,7 +29030,7 @@
         <v>0</v>
       </c>
       <c r="D952" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E952" t="n">
         <v>6.772908366533864</v>
@@ -29066,7 +29057,7 @@
         <v>59.36254980079681</v>
       </c>
       <c r="C953" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="D953" t="n">
         <v>19.9203187250996</v>
@@ -29129,7 +29120,7 @@
         <v>6.374501992031881</v>
       </c>
       <c r="D955" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E955" t="n">
         <v>59.36254980079681</v>
@@ -29159,7 +29150,7 @@
         <v>8.366533864541836</v>
       </c>
       <c r="D956" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E956" t="n">
         <v>76.09561752988047</v>
@@ -29189,7 +29180,7 @@
         <v>8.366533864541836</v>
       </c>
       <c r="D957" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E957" t="n">
         <v>97.60956175298804</v>
@@ -29219,7 +29210,7 @@
         <v>9.561752988047814</v>
       </c>
       <c r="D958" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E958" t="n">
         <v>96.81274900398408</v>
@@ -29249,7 +29240,7 @@
         <v>20.7171314741036</v>
       </c>
       <c r="D959" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E959" t="n">
         <v>93.62549800796812</v>
@@ -29279,7 +29270,7 @@
         <v>24.30278884462152</v>
       </c>
       <c r="D960" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E960" t="n">
         <v>94.82071713147413</v>
@@ -29288,7 +29279,7 @@
         <v>86.45418326693228</v>
       </c>
       <c r="G960" t="n">
-        <v>56.25498007968127</v>
+        <v>56.25498007968128</v>
       </c>
       <c r="H960" s="4" t="inlineStr">
         <is>
@@ -29309,7 +29300,7 @@
         <v>33.06772908366534</v>
       </c>
       <c r="D961" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E961" t="n">
         <v>97.21115537848604</v>
@@ -29339,7 +29330,7 @@
         <v>39.8406374501992</v>
       </c>
       <c r="D962" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E962" t="n">
         <v>94.82071713147413</v>
@@ -29369,7 +29360,7 @@
         <v>38.24701195219124</v>
       </c>
       <c r="D963" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E963" t="n">
         <v>97.60956175298804</v>
@@ -29399,7 +29390,7 @@
         <v>31.07569721115537</v>
       </c>
       <c r="D964" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E964" t="n">
         <v>74.90039840637451</v>
@@ -29429,7 +29420,7 @@
         <v>35.85657370517929</v>
       </c>
       <c r="D965" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E965" t="n">
         <v>68.12749003984064</v>
@@ -29459,7 +29450,7 @@
         <v>37.05179282868526</v>
       </c>
       <c r="D966" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E966" t="n">
         <v>48.60557768924303</v>
@@ -29489,7 +29480,7 @@
         <v>27.09163346613546</v>
       </c>
       <c r="D967" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E967" t="n">
         <v>56.97211155378486</v>
@@ -29519,7 +29510,7 @@
         <v>25.4980079681275</v>
       </c>
       <c r="D968" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E968" t="n">
         <v>51.79282868525896</v>
@@ -29549,7 +29540,7 @@
         <v>27.88844621513944</v>
       </c>
       <c r="D969" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E969" t="n">
         <v>46.61354581673307</v>
@@ -29579,7 +29570,7 @@
         <v>26.29482071713147</v>
       </c>
       <c r="D970" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E970" t="n">
         <v>68.12749003984064</v>
@@ -29609,7 +29600,7 @@
         <v>31.07569721115537</v>
       </c>
       <c r="D971" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E971" t="n">
         <v>64.14342629482071</v>
@@ -29639,7 +29630,7 @@
         <v>31.07569721115537</v>
       </c>
       <c r="D972" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E972" t="n">
         <v>73.70517928286853</v>
@@ -29669,7 +29660,7 @@
         <v>34.66135458167331</v>
       </c>
       <c r="D973" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E973" t="n">
         <v>58.96414342629483</v>
@@ -29699,7 +29690,7 @@
         <v>39.8406374501992</v>
       </c>
       <c r="D974" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E974" t="n">
         <v>82.47011952191235</v>
@@ -29729,7 +29720,7 @@
         <v>43.42629482071712</v>
       </c>
       <c r="D975" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E975" t="n">
         <v>66.13545816733067</v>
@@ -29759,7 +29750,7 @@
         <v>47.80876494023904</v>
       </c>
       <c r="D976" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E976" t="n">
         <v>84.46215139442231</v>
@@ -29789,7 +29780,7 @@
         <v>35.85657370517929</v>
       </c>
       <c r="D977" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E977" t="n">
         <v>71.71314741035857</v>
@@ -29819,7 +29810,7 @@
         <v>26.29482071713147</v>
       </c>
       <c r="D978" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E978" t="n">
         <v>82.47011952191235</v>
@@ -29849,7 +29840,7 @@
         <v>24.30278884462152</v>
       </c>
       <c r="D979" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E979" t="n">
         <v>73.30677290836654</v>
@@ -29876,10 +29867,10 @@
         <v>94.02390438247012</v>
       </c>
       <c r="C980" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D980" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E980" t="n">
         <v>60.95617529880478</v>
@@ -29888,7 +29879,7 @@
         <v>78.48605577689243</v>
       </c>
       <c r="G980" t="n">
-        <v>56.73306772908366</v>
+        <v>56.73306772908367</v>
       </c>
       <c r="H980" s="4" t="inlineStr">
         <is>
@@ -29909,7 +29900,7 @@
         <v>34.26294820717132</v>
       </c>
       <c r="D981" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E981" t="n">
         <v>76.89243027888446</v>
@@ -29939,7 +29930,7 @@
         <v>27.09163346613546</v>
       </c>
       <c r="D982" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E982" t="n">
         <v>85.65737051792829</v>
@@ -29969,7 +29960,7 @@
         <v>27.09163346613546</v>
       </c>
       <c r="D983" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E983" t="n">
         <v>85.65737051792829</v>
@@ -29978,7 +29969,7 @@
         <v>80.47808764940238</v>
       </c>
       <c r="G983" t="n">
-        <v>62.62948207171315</v>
+        <v>62.62948207171316</v>
       </c>
       <c r="H983" s="4" t="inlineStr">
         <is>
@@ -29999,7 +29990,7 @@
         <v>22.70916334661355</v>
       </c>
       <c r="D984" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E984" t="n">
         <v>89.64143426294821</v>
@@ -30029,7 +30020,7 @@
         <v>20.7171314741036</v>
       </c>
       <c r="D985" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E985" t="n">
         <v>41.83266932270917</v>
@@ -30059,7 +30050,7 @@
         <v>17.13147410358566</v>
       </c>
       <c r="D986" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="E986" t="n">
         <v>51.39442231075697</v>
@@ -30068,7 +30059,7 @@
         <v>78.48605577689243</v>
       </c>
       <c r="G986" t="n">
-        <v>52.11155378486055</v>
+        <v>52.11155378486056</v>
       </c>
       <c r="H986" s="3" t="inlineStr">
         <is>
@@ -30638,7 +30629,7 @@
         <v>25.89641434262948</v>
       </c>
       <c r="G1005" t="n">
-        <v>41.99203187250995</v>
+        <v>41.99203187250996</v>
       </c>
       <c r="H1005" s="2" t="inlineStr">
         <is>
@@ -30815,7 +30806,7 @@
         <v>45.81673306772908</v>
       </c>
       <c r="F1011" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="G1011" t="n">
         <v>45.1792828685259</v>
@@ -30848,7 +30839,7 @@
         <v>35.85657370517929</v>
       </c>
       <c r="G1012" t="n">
-        <v>47.96812749003983</v>
+        <v>47.96812749003984</v>
       </c>
       <c r="H1012" s="3" t="inlineStr">
         <is>
@@ -31508,7 +31499,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="G1034" t="n">
-        <v>56.25498007968127</v>
+        <v>56.25498007968128</v>
       </c>
       <c r="H1034" s="4" t="inlineStr">
         <is>
@@ -31625,7 +31616,7 @@
         <v>1.195219123505976</v>
       </c>
       <c r="F1038" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G1038" t="n">
         <v>15.45816733067729</v>
@@ -31655,7 +31646,7 @@
         <v>8.764940239043826</v>
       </c>
       <c r="F1039" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G1039" t="n">
         <v>21.51394422310757</v>
@@ -31673,7 +31664,7 @@
         </is>
       </c>
       <c r="B1040" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C1040" t="n">
         <v>36.65338645418327</v>
@@ -31736,7 +31727,7 @@
         <v>25.0996015936255</v>
       </c>
       <c r="C1042" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="D1042" t="n">
         <v>16.33466135458167</v>
@@ -31823,7 +31814,7 @@
         </is>
       </c>
       <c r="B1045" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="C1045" t="n">
         <v>60.95617529880478</v>
@@ -32282,7 +32273,7 @@
         <v>3.585657370517929</v>
       </c>
       <c r="E1060" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F1060" t="n">
         <v>4.382470119521913</v>
@@ -32555,10 +32546,10 @@
         <v>64.5418326693227</v>
       </c>
       <c r="F1069" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G1069" t="n">
-        <v>28.28685258964143</v>
+        <v>28.28685258964144</v>
       </c>
       <c r="H1069" s="2" t="inlineStr">
         <is>
@@ -32786,7 +32777,7 @@
         <v>10.35856573705179</v>
       </c>
       <c r="C1077" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="D1077" t="n">
         <v>22.70916334661354</v>
@@ -33428,7 +33419,7 @@
         <v>5.577689243027888</v>
       </c>
       <c r="G1098" t="n">
-        <v>22.54980079681275</v>
+        <v>22.54980079681276</v>
       </c>
       <c r="H1098" s="6" t="inlineStr">
         <is>
@@ -33602,7 +33593,7 @@
         <v>0</v>
       </c>
       <c r="E1104" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="F1104" t="n">
         <v>6.374501992031872</v>
@@ -33968,7 +33959,7 @@
         <v>15.53784860557769</v>
       </c>
       <c r="G1116" t="n">
-        <v>29.24302788844622</v>
+        <v>29.24302788844621</v>
       </c>
       <c r="H1116" s="2" t="inlineStr">
         <is>
@@ -34175,7 +34166,7 @@
         <v>7.171314741035857</v>
       </c>
       <c r="F1123" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G1123" t="n">
         <v>14.66135458167331</v>
@@ -34232,7 +34223,7 @@
         <v>34.26294820717131</v>
       </c>
       <c r="E1125" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="F1125" t="n">
         <v>31.87250996015936</v>
@@ -34292,7 +34283,7 @@
         <v>0</v>
       </c>
       <c r="E1127" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F1127" t="n">
         <v>37.84860557768924</v>
@@ -34772,7 +34763,7 @@
         <v>0</v>
       </c>
       <c r="E1143" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F1143" t="n">
         <v>18.72509960159363</v>
@@ -34835,7 +34826,7 @@
         <v>36.65338645418327</v>
       </c>
       <c r="F1145" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="G1145" t="n">
         <v>31.15537848605578</v>
@@ -35123,7 +35114,7 @@
         </is>
       </c>
       <c r="B1155" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C1155" t="n">
         <v>59.36254980079681</v>
@@ -35498,7 +35489,7 @@
         <v>80.47808764940238</v>
       </c>
       <c r="G1167" t="n">
-        <v>60.07968127490039</v>
+        <v>60.0796812749004</v>
       </c>
       <c r="H1167" s="4" t="inlineStr">
         <is>
@@ -35708,7 +35699,7 @@
         <v>67.72908366533864</v>
       </c>
       <c r="G1174" t="n">
-        <v>44.46215139442231</v>
+        <v>44.46215139442232</v>
       </c>
       <c r="H1174" s="2" t="inlineStr">
         <is>
@@ -35846,7 +35837,7 @@
         <v>49.00398406374502</v>
       </c>
       <c r="C1179" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="D1179" t="n">
         <v>17.92828685258964</v>
@@ -35948,7 +35939,7 @@
         <v>98.40637450199203</v>
       </c>
       <c r="G1182" t="n">
-        <v>50.27888446215139</v>
+        <v>50.2788844621514</v>
       </c>
       <c r="H1182" s="3" t="inlineStr">
         <is>
@@ -36068,7 +36059,7 @@
         <v>64.5418326693227</v>
       </c>
       <c r="G1186" t="n">
-        <v>38.16733067729083</v>
+        <v>38.16733067729084</v>
       </c>
       <c r="H1186" s="2" t="inlineStr">
         <is>
@@ -36098,7 +36089,7 @@
         <v>66.13545816733067</v>
       </c>
       <c r="G1187" t="n">
-        <v>48.28685258964143</v>
+        <v>48.28685258964144</v>
       </c>
       <c r="H1187" s="3" t="inlineStr">
         <is>
@@ -36302,7 +36293,7 @@
         <v>17.52988047808765</v>
       </c>
       <c r="E1194" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="F1194" t="n">
         <v>56.17529880478087</v>
@@ -36416,7 +36407,7 @@
         <v>61.35458167330678</v>
       </c>
       <c r="C1198" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="D1198" t="n">
         <v>17.52988047808765</v>
@@ -36428,7 +36419,7 @@
         <v>57.76892430278885</v>
       </c>
       <c r="G1198" t="n">
-        <v>40.55776892430278</v>
+        <v>40.55776892430279</v>
       </c>
       <c r="H1198" s="2" t="inlineStr">
         <is>
@@ -36458,7 +36449,7 @@
         <v>79.2828685258964</v>
       </c>
       <c r="G1199" t="n">
-        <v>60.55776892430278</v>
+        <v>60.55776892430279</v>
       </c>
       <c r="H1199" s="4" t="inlineStr">
         <is>
@@ -37328,7 +37319,7 @@
         <v>60.95617529880478</v>
       </c>
       <c r="G1228" t="n">
-        <v>60.63745019920319</v>
+        <v>60.6374501992032</v>
       </c>
       <c r="H1228" s="4" t="inlineStr">
         <is>
@@ -37592,7 +37583,7 @@
         <v>18.72509960159363</v>
       </c>
       <c r="E1237" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F1237" t="n">
         <v>29.8804780876494</v>
@@ -37778,7 +37769,7 @@
         <v>26.29482071713147</v>
       </c>
       <c r="G1243" t="n">
-        <v>52.43027888446215</v>
+        <v>52.43027888446216</v>
       </c>
       <c r="H1243" s="3" t="inlineStr">
         <is>
@@ -39938,7 +39929,7 @@
         <v>47.80876494023904</v>
       </c>
       <c r="G1315" t="n">
-        <v>50.27888446215139</v>
+        <v>50.2788844621514</v>
       </c>
       <c r="H1315" s="3" t="inlineStr">
         <is>
@@ -40058,7 +40049,7 @@
         <v>48.20717131474104</v>
       </c>
       <c r="G1319" t="n">
-        <v>60.07968127490039</v>
+        <v>60.0796812749004</v>
       </c>
       <c r="H1319" s="4" t="inlineStr">
         <is>
@@ -40298,7 +40289,7 @@
         <v>43.82470119521912</v>
       </c>
       <c r="G1327" t="n">
-        <v>44.3824701195219</v>
+        <v>44.38247011952191</v>
       </c>
       <c r="H1327" s="2" t="inlineStr">
         <is>
@@ -40985,7 +40976,7 @@
         <v>22.70916334661354</v>
       </c>
       <c r="F1350" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G1350" t="n">
         <v>39.68127490039841</v>
@@ -41033,7 +41024,7 @@
         </is>
       </c>
       <c r="B1352" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C1352" t="n">
         <v>62.15139442231076</v>
@@ -41063,7 +41054,7 @@
         </is>
       </c>
       <c r="B1353" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="C1353" t="n">
         <v>44.22310756972112</v>
@@ -41123,7 +41114,7 @@
         </is>
       </c>
       <c r="B1355" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C1355" t="n">
         <v>40.63745019920319</v>
@@ -41153,7 +41144,7 @@
         </is>
       </c>
       <c r="B1356" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="C1356" t="n">
         <v>28.28685258964143</v>
@@ -41423,7 +41414,7 @@
         </is>
       </c>
       <c r="B1365" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C1365" t="n">
         <v>61.35458167330678</v>
@@ -41585,7 +41576,7 @@
         <v>21.91235059760956</v>
       </c>
       <c r="F1370" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G1370" t="n">
         <v>23.74501992031873</v>
@@ -42482,7 +42473,7 @@
         <v>13.14741035856574</v>
       </c>
       <c r="E1400" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F1400" t="n">
         <v>4.382470119521913</v>
@@ -42776,7 +42767,7 @@
         <v>11.55378486055777</v>
       </c>
       <c r="C1410" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D1410" t="n">
         <v>43.02788844621514</v>
@@ -42848,7 +42839,7 @@
         <v>93.22709163346612</v>
       </c>
       <c r="G1412" t="n">
-        <v>52.11155378486055</v>
+        <v>52.11155378486056</v>
       </c>
       <c r="H1412" s="3" t="inlineStr">
         <is>
@@ -43382,7 +43373,7 @@
         <v>45.0199203187251</v>
       </c>
       <c r="E1430" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F1430" t="n">
         <v>19.9203187250996</v>
@@ -44123,7 +44114,7 @@
         </is>
       </c>
       <c r="B1455" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C1455" t="n">
         <v>31.87250996015936</v>
@@ -44648,7 +44639,7 @@
         <v>41.03585657370518</v>
       </c>
       <c r="G1472" t="n">
-        <v>50.27888446215139</v>
+        <v>50.2788844621514</v>
       </c>
       <c r="H1472" s="3" t="inlineStr">
         <is>
@@ -44738,7 +44729,7 @@
         <v>46.61354581673307</v>
       </c>
       <c r="G1475" t="n">
-        <v>48.28685258964143</v>
+        <v>48.28685258964144</v>
       </c>
       <c r="H1475" s="3" t="inlineStr">
         <is>
@@ -44786,7 +44777,7 @@
         <v>31.87250996015936</v>
       </c>
       <c r="C1477" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D1477" t="n">
         <v>17.52988047808765</v>
@@ -44846,7 +44837,7 @@
         <v>37.84860557768924</v>
       </c>
       <c r="C1479" t="n">
-        <v>46.61354581673307</v>
+        <v>47.01195219123506</v>
       </c>
       <c r="D1479" t="n">
         <v>35.45816733067729</v>
@@ -44858,11 +44849,71 @@
         <v>63.74501992031873</v>
       </c>
       <c r="G1479" t="n">
-        <v>54.10358565737051</v>
+        <v>54.18326693227092</v>
       </c>
       <c r="H1479" s="3" t="inlineStr">
         <is>
           <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B1480" t="n">
+        <v>47.01195219123506</v>
+      </c>
+      <c r="C1480" t="n">
+        <v>57.37051792828685</v>
+      </c>
+      <c r="D1480" t="n">
+        <v>43.82470119521912</v>
+      </c>
+      <c r="E1480" t="n">
+        <v>94.42231075697212</v>
+      </c>
+      <c r="F1480" t="n">
+        <v>68.12749003984064</v>
+      </c>
+      <c r="G1480" t="n">
+        <v>62.15139442231075</v>
+      </c>
+      <c r="H1480" s="4" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B1481" t="n">
+        <v>49.00398406374502</v>
+      </c>
+      <c r="C1481" t="n">
+        <v>54.18326693227092</v>
+      </c>
+      <c r="D1481" t="n">
+        <v>43.42629482071713</v>
+      </c>
+      <c r="E1481" t="n">
+        <v>92.03187250996017</v>
+      </c>
+      <c r="F1481" t="n">
+        <v>58.96414342629483</v>
+      </c>
+      <c r="G1481" t="n">
+        <v>59.52191235059761</v>
+      </c>
+      <c r="H1481" s="4" t="inlineStr">
+        <is>
+          <t>Greed</t>
         </is>
       </c>
     </row>
@@ -44877,7 +44928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I278"/>
+  <dimension ref="A1:I281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46019,7 +46070,7 @@
         <v>96.41434262948206</v>
       </c>
       <c r="H34" t="n">
-        <v>45.94953519256307</v>
+        <v>45.94953519256308</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -46109,7 +46160,7 @@
         <v>18.72509960159363</v>
       </c>
       <c r="E37" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F37" t="n">
         <v>29.8804780876494</v>
@@ -46379,7 +46430,7 @@
         <v>39.44223107569721</v>
       </c>
       <c r="G45" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="H45" t="n">
         <v>47.60956175298804</v>
@@ -46940,7 +46991,7 @@
         <v>66.13545816733067</v>
       </c>
       <c r="G62" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="H62" t="n">
         <v>64.01062416998673</v>
@@ -47504,7 +47555,7 @@
         <v>62.15139442231076</v>
       </c>
       <c r="H79" t="n">
-        <v>50.33200531208499</v>
+        <v>50.332005312085</v>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
@@ -47636,7 +47687,7 @@
         <v>23.90438247011953</v>
       </c>
       <c r="H83" t="n">
-        <v>60.55776892430278</v>
+        <v>60.55776892430279</v>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
@@ -47768,7 +47819,7 @@
         <v>23.90438247011953</v>
       </c>
       <c r="H87" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="I87" s="4" t="inlineStr">
         <is>
@@ -48560,7 +48611,7 @@
         <v>43.82470119521913</v>
       </c>
       <c r="H111" t="n">
-        <v>56.44090305444887</v>
+        <v>56.44090305444888</v>
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
@@ -48590,7 +48641,7 @@
         <v>50.59760956175299</v>
       </c>
       <c r="G112" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="H112" t="n">
         <v>52.65604249667995</v>
@@ -48791,7 +48842,7 @@
         <v>12.35059760956176</v>
       </c>
       <c r="H118" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I118" s="3" t="inlineStr">
         <is>
@@ -48923,7 +48974,7 @@
         <v>64.9402390438247</v>
       </c>
       <c r="H122" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I122" s="3" t="inlineStr">
         <is>
@@ -49121,7 +49172,7 @@
         <v>43.82470119521913</v>
       </c>
       <c r="H128" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
@@ -49415,7 +49466,7 @@
         <v>40.23904382470119</v>
       </c>
       <c r="G137" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="H137" t="n">
         <v>60.02656042496679</v>
@@ -49550,7 +49601,7 @@
         <v>5.179282868525888</v>
       </c>
       <c r="H141" t="n">
-        <v>53.91766268260291</v>
+        <v>53.91766268260292</v>
       </c>
       <c r="I141" s="3" t="inlineStr">
         <is>
@@ -49715,7 +49766,7 @@
         <v>97.60956175298804</v>
       </c>
       <c r="H146" t="n">
-        <v>50.13280212483399</v>
+        <v>50.132802124834</v>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
@@ -49841,7 +49892,7 @@
         <v>22.70916334661354</v>
       </c>
       <c r="F150" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G150" t="n">
         <v>74.10358565737052</v>
@@ -49895,7 +49946,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C152" t="n">
         <v>62.15139442231076</v>
@@ -49928,7 +49979,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="C153" t="n">
         <v>44.22310756972112</v>
@@ -49979,7 +50030,7 @@
         <v>78.48605577689243</v>
       </c>
       <c r="H154" t="n">
-        <v>23.17397078353254</v>
+        <v>23.17397078353253</v>
       </c>
       <c r="I154" s="6" t="inlineStr">
         <is>
@@ -49994,7 +50045,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C155" t="n">
         <v>40.63745019920319</v>
@@ -50027,7 +50078,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="C156" t="n">
         <v>28.28685258964143</v>
@@ -50324,7 +50375,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C165" t="n">
         <v>61.35458167330678</v>
@@ -50501,7 +50552,7 @@
         <v>21.91235059760956</v>
       </c>
       <c r="F170" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G170" t="n">
         <v>97.60956175298804</v>
@@ -50702,7 +50753,7 @@
         <v>82.47011952191235</v>
       </c>
       <c r="G176" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="H176" t="n">
         <v>45.08632138114209</v>
@@ -51488,7 +51539,7 @@
         <v>13.14741035856574</v>
       </c>
       <c r="E200" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F200" t="n">
         <v>4.382470119521913</v>
@@ -51794,7 +51845,7 @@
         <v>39.44223107569721</v>
       </c>
       <c r="H209" t="n">
-        <v>50.33200531208499</v>
+        <v>50.332005312085</v>
       </c>
       <c r="I209" s="3" t="inlineStr">
         <is>
@@ -51812,7 +51863,7 @@
         <v>11.55378486055777</v>
       </c>
       <c r="C210" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D210" t="n">
         <v>43.02788844621514</v>
@@ -52322,7 +52373,7 @@
         <v>87.25099601593625</v>
       </c>
       <c r="H225" t="n">
-        <v>36.12217795484727</v>
+        <v>36.12217795484728</v>
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
@@ -52478,7 +52529,7 @@
         <v>45.0199203187251</v>
       </c>
       <c r="E230" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F230" t="n">
         <v>19.9203187250996</v>
@@ -53294,7 +53345,7 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C255" t="n">
         <v>31.87250996015936</v>
@@ -54023,7 +54074,7 @@
         <v>31.87250996015936</v>
       </c>
       <c r="C277" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D277" t="n">
         <v>17.52988047808765</v>
@@ -54074,6 +54125,105 @@
         <v>46.61354581673307</v>
       </c>
       <c r="I278" s="3" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>37.84860557768924</v>
+      </c>
+      <c r="C279" t="n">
+        <v>47.01195219123506</v>
+      </c>
+      <c r="D279" t="n">
+        <v>35.45816733067729</v>
+      </c>
+      <c r="E279" t="n">
+        <v>86.85258964143426</v>
+      </c>
+      <c r="F279" t="n">
+        <v>63.74501992031873</v>
+      </c>
+      <c r="G279" t="n">
+        <v>44.62151394422311</v>
+      </c>
+      <c r="H279" t="n">
+        <v>52.58964143426295</v>
+      </c>
+      <c r="I279" s="3" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>47.01195219123506</v>
+      </c>
+      <c r="C280" t="n">
+        <v>57.37051792828685</v>
+      </c>
+      <c r="D280" t="n">
+        <v>43.82470119521912</v>
+      </c>
+      <c r="E280" t="n">
+        <v>94.42231075697212</v>
+      </c>
+      <c r="F280" t="n">
+        <v>68.12749003984064</v>
+      </c>
+      <c r="G280" t="n">
+        <v>14.7410358565737</v>
+      </c>
+      <c r="H280" t="n">
+        <v>54.24966799468791</v>
+      </c>
+      <c r="I280" s="3" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>49.00398406374502</v>
+      </c>
+      <c r="C281" t="n">
+        <v>54.18326693227092</v>
+      </c>
+      <c r="D281" t="n">
+        <v>43.42629482071713</v>
+      </c>
+      <c r="E281" t="n">
+        <v>92.03187250996017</v>
+      </c>
+      <c r="F281" t="n">
+        <v>58.96414342629483</v>
+      </c>
+      <c r="G281" t="n">
+        <v>8.366533864541836</v>
+      </c>
+      <c r="H281" t="n">
+        <v>50.99601593625498</v>
+      </c>
+      <c r="I281" s="3" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
@@ -54117,7 +54267,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-30 17:36 UTC</t>
+          <t>2026-07-30 17:39 UTC</t>
         </is>
       </c>
     </row>
@@ -54129,7 +54279,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1478 days, 2020-06-11 to 2026-07-28</t>
+          <t>1480 days, 2020-06-11 to 2026-07-30</t>
         </is>
       </c>
     </row>
@@ -54141,7 +54291,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>277 days, 2025-06-11 to 2026-07-27</t>
+          <t>280 days, 2025-06-11 to 2026-07-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-07-31
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1481"/>
+  <dimension ref="A1:H1482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44917,6 +44917,36 @@
         </is>
       </c>
     </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B1482" t="n">
+        <v>52.58964143426294</v>
+      </c>
+      <c r="C1482" t="n">
+        <v>65.33864541832669</v>
+      </c>
+      <c r="D1482" t="n">
+        <v>43.02788844621514</v>
+      </c>
+      <c r="E1482" t="n">
+        <v>94.42231075697212</v>
+      </c>
+      <c r="F1482" t="n">
+        <v>64.14342629482071</v>
+      </c>
+      <c r="G1482" t="n">
+        <v>63.90438247011952</v>
+      </c>
+      <c r="H1482" s="4" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -44928,7 +44958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I281"/>
+  <dimension ref="A1:I282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54224,6 +54254,39 @@
         <v>50.99601593625498</v>
       </c>
       <c r="I281" s="3" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>52.58964143426294</v>
+      </c>
+      <c r="C282" t="n">
+        <v>65.33864541832669</v>
+      </c>
+      <c r="D282" t="n">
+        <v>43.02788844621514</v>
+      </c>
+      <c r="E282" t="n">
+        <v>94.42231075697212</v>
+      </c>
+      <c r="F282" t="n">
+        <v>64.14342629482071</v>
+      </c>
+      <c r="G282" t="n">
+        <v>2.788844621513945</v>
+      </c>
+      <c r="H282" t="n">
+        <v>53.71845949535192</v>
+      </c>
+      <c r="I282" s="3" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
@@ -54267,7 +54330,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-30 17:39 UTC</t>
+          <t>2026-07-31 14:45 UTC</t>
         </is>
       </c>
     </row>
@@ -54279,7 +54342,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1480 days, 2020-06-11 to 2026-07-30</t>
+          <t>1481 days, 2020-06-11 to 2026-07-31</t>
         </is>
       </c>
     </row>
@@ -54291,7 +54354,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>280 days, 2025-06-11 to 2026-07-30</t>
+          <t>281 days, 2025-06-11 to 2026-07-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-08-01
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -44933,13 +44933,13 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E1482" t="n">
-        <v>94.42231075697212</v>
+        <v>92.03187250996017</v>
       </c>
       <c r="F1482" t="n">
         <v>64.14342629482071</v>
       </c>
       <c r="G1482" t="n">
-        <v>63.90438247011952</v>
+        <v>63.42629482071712</v>
       </c>
       <c r="H1482" s="4" t="inlineStr">
         <is>
@@ -54275,7 +54275,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>94.42231075697212</v>
+        <v>92.03187250996017</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -54284,7 +54284,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.71845949535192</v>
+        <v>53.32005312084993</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -54330,7 +54330,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-31 14:45 UTC</t>
+          <t>2026-08-01 14:04 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-08-02
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -44933,13 +44933,13 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E1482" t="n">
-        <v>92.03187250996017</v>
+        <v>94.42231075697212</v>
       </c>
       <c r="F1482" t="n">
         <v>64.14342629482071</v>
       </c>
       <c r="G1482" t="n">
-        <v>63.42629482071712</v>
+        <v>63.90438247011952</v>
       </c>
       <c r="H1482" s="4" t="inlineStr">
         <is>
@@ -54275,7 +54275,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>92.03187250996017</v>
+        <v>94.42231075697212</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -54284,7 +54284,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.32005312084993</v>
+        <v>53.71845949535192</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -54330,7 +54330,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-01 14:04 UTC</t>
+          <t>2026-08-02 14:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-08-03
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1482"/>
+  <dimension ref="A1:H1483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44947,6 +44947,36 @@
         </is>
       </c>
     </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B1483" t="n">
+        <v>75.69721115537848</v>
+      </c>
+      <c r="C1483" t="n">
+        <v>61.75298804780876</v>
+      </c>
+      <c r="D1483" t="n">
+        <v>42.62948207171315</v>
+      </c>
+      <c r="E1483" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1483" t="n">
+        <v>81.67330677290838</v>
+      </c>
+      <c r="G1483" t="n">
+        <v>72.35059760956176</v>
+      </c>
+      <c r="H1483" s="4" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -44958,7 +44988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I282"/>
+  <dimension ref="A1:I283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54289,6 +54319,39 @@
       <c r="I282" s="3" t="inlineStr">
         <is>
           <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>75.69721115537848</v>
+      </c>
+      <c r="C283" t="n">
+        <v>61.75298804780876</v>
+      </c>
+      <c r="D283" t="n">
+        <v>42.62948207171315</v>
+      </c>
+      <c r="E283" t="n">
+        <v>100</v>
+      </c>
+      <c r="F283" t="n">
+        <v>81.67330677290838</v>
+      </c>
+      <c r="G283" t="n">
+        <v>2.788844621513945</v>
+      </c>
+      <c r="H283" t="n">
+        <v>60.75697211155379</v>
+      </c>
+      <c r="I283" s="4" t="inlineStr">
+        <is>
+          <t>Greed</t>
         </is>
       </c>
     </row>
@@ -54330,7 +54393,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-02 14:06 UTC</t>
+          <t>2026-08-03 15:23 UTC</t>
         </is>
       </c>
     </row>
@@ -54342,7 +54405,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1481 days, 2020-06-11 to 2026-07-31</t>
+          <t>1482 days, 2020-06-11 to 2026-08-03</t>
         </is>
       </c>
     </row>
@@ -54354,7 +54417,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>281 days, 2025-06-11 to 2026-07-31</t>
+          <t>282 days, 2025-06-11 to 2026-08-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-08-04
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Core" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Core" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Extended" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -77,7 +74,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -85,19 +82,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -105,7 +96,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I283"/>
+  <dimension ref="A1:I284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1604,7 @@
         <v>96.41434262948206</v>
       </c>
       <c r="H34" t="n">
-        <v>45.94953519256307</v>
+        <v>45.94953519256308</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -1703,7 +1694,7 @@
         <v>18.72509960159363</v>
       </c>
       <c r="E37" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F37" t="n">
         <v>29.8804780876494</v>
@@ -1973,7 +1964,7 @@
         <v>39.44223107569721</v>
       </c>
       <c r="G45" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="H45" t="n">
         <v>47.60956175298804</v>
@@ -2534,7 +2525,7 @@
         <v>66.13545816733067</v>
       </c>
       <c r="G62" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="H62" t="n">
         <v>64.01062416998673</v>
@@ -3098,7 +3089,7 @@
         <v>62.15139442231076</v>
       </c>
       <c r="H79" t="n">
-        <v>50.33200531208499</v>
+        <v>50.332005312085</v>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
@@ -3230,7 +3221,7 @@
         <v>23.90438247011953</v>
       </c>
       <c r="H83" t="n">
-        <v>60.55776892430278</v>
+        <v>60.55776892430279</v>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
@@ -3362,7 +3353,7 @@
         <v>23.90438247011953</v>
       </c>
       <c r="H87" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
@@ -4154,7 +4145,7 @@
         <v>43.82470119521913</v>
       </c>
       <c r="H111" t="n">
-        <v>56.44090305444887</v>
+        <v>56.44090305444888</v>
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
@@ -4184,7 +4175,7 @@
         <v>50.59760956175299</v>
       </c>
       <c r="G112" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="H112" t="n">
         <v>52.65604249667995</v>
@@ -4385,7 +4376,7 @@
         <v>12.35059760956176</v>
       </c>
       <c r="H118" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I118" s="3" t="inlineStr">
         <is>
@@ -4517,7 +4508,7 @@
         <v>64.9402390438247</v>
       </c>
       <c r="H122" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I122" s="3" t="inlineStr">
         <is>
@@ -4715,7 +4706,7 @@
         <v>43.82470119521913</v>
       </c>
       <c r="H128" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
@@ -5009,7 +5000,7 @@
         <v>40.23904382470119</v>
       </c>
       <c r="G137" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="H137" t="n">
         <v>60.02656042496679</v>
@@ -5144,7 +5135,7 @@
         <v>5.179282868525888</v>
       </c>
       <c r="H141" t="n">
-        <v>53.91766268260291</v>
+        <v>53.91766268260292</v>
       </c>
       <c r="I141" s="3" t="inlineStr">
         <is>
@@ -5309,7 +5300,7 @@
         <v>97.60956175298804</v>
       </c>
       <c r="H146" t="n">
-        <v>50.13280212483399</v>
+        <v>50.132802124834</v>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
@@ -5435,7 +5426,7 @@
         <v>22.70916334661354</v>
       </c>
       <c r="F150" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G150" t="n">
         <v>74.10358565737052</v>
@@ -5489,7 +5480,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C152" t="n">
         <v>62.15139442231076</v>
@@ -5522,7 +5513,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="C153" t="n">
         <v>44.22310756972112</v>
@@ -5573,7 +5564,7 @@
         <v>78.48605577689243</v>
       </c>
       <c r="H154" t="n">
-        <v>23.17397078353254</v>
+        <v>23.17397078353253</v>
       </c>
       <c r="I154" s="6" t="inlineStr">
         <is>
@@ -5588,7 +5579,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C155" t="n">
         <v>40.63745019920319</v>
@@ -5621,7 +5612,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="C156" t="n">
         <v>28.28685258964143</v>
@@ -5918,7 +5909,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C165" t="n">
         <v>61.35458167330678</v>
@@ -6095,7 +6086,7 @@
         <v>21.91235059760956</v>
       </c>
       <c r="F170" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G170" t="n">
         <v>97.60956175298804</v>
@@ -6296,7 +6287,7 @@
         <v>82.47011952191235</v>
       </c>
       <c r="G176" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="H176" t="n">
         <v>45.08632138114209</v>
@@ -7082,7 +7073,7 @@
         <v>13.14741035856574</v>
       </c>
       <c r="E200" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F200" t="n">
         <v>4.382470119521913</v>
@@ -7388,7 +7379,7 @@
         <v>39.44223107569721</v>
       </c>
       <c r="H209" t="n">
-        <v>50.33200531208499</v>
+        <v>50.332005312085</v>
       </c>
       <c r="I209" s="3" t="inlineStr">
         <is>
@@ -7406,7 +7397,7 @@
         <v>11.55378486055777</v>
       </c>
       <c r="C210" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D210" t="n">
         <v>43.02788844621514</v>
@@ -7916,7 +7907,7 @@
         <v>87.25099601593625</v>
       </c>
       <c r="H225" t="n">
-        <v>36.12217795484727</v>
+        <v>36.12217795484728</v>
       </c>
       <c r="I225" s="4" t="inlineStr">
         <is>
@@ -8072,7 +8063,7 @@
         <v>45.0199203187251</v>
       </c>
       <c r="E230" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F230" t="n">
         <v>19.9203187250996</v>
@@ -8888,7 +8879,7 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C255" t="n">
         <v>31.87250996015936</v>
@@ -9617,7 +9608,7 @@
         <v>31.87250996015936</v>
       </c>
       <c r="C277" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D277" t="n">
         <v>17.52988047808765</v>
@@ -9788,7 +9779,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>92.03187250996017</v>
+        <v>94.42231075697212</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -9797,7 +9788,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.32005312084993</v>
+        <v>53.71845949535192</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -9821,7 +9812,7 @@
         <v>42.62948207171315</v>
       </c>
       <c r="E283" t="n">
-        <v>98.80478087649402</v>
+        <v>100</v>
       </c>
       <c r="F283" t="n">
         <v>81.67330677290838</v>
@@ -9830,9 +9821,42 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H283" t="n">
-        <v>60.55776892430278</v>
+        <v>60.75697211155379</v>
       </c>
       <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>68.12749003984064</v>
+      </c>
+      <c r="C284" t="n">
+        <v>52.98804780876494</v>
+      </c>
+      <c r="D284" t="n">
+        <v>35.85657370517929</v>
+      </c>
+      <c r="E284" t="n">
+        <v>90.0398406374502</v>
+      </c>
+      <c r="F284" t="n">
+        <v>78.88446215139442</v>
+      </c>
+      <c r="G284" t="n">
+        <v>44.62151394422311</v>
+      </c>
+      <c r="H284" t="n">
+        <v>61.75298804780877</v>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
         <is>
           <t>Greed</t>
         </is>
@@ -9849,7 +9873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I283"/>
+  <dimension ref="A1:I284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10991,7 +11015,7 @@
         <v>96.41434262948206</v>
       </c>
       <c r="H34" t="n">
-        <v>45.94953519256307</v>
+        <v>45.94953519256308</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
@@ -11081,7 +11105,7 @@
         <v>18.72509960159363</v>
       </c>
       <c r="E37" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F37" t="n">
         <v>29.8804780876494</v>
@@ -11351,7 +11375,7 @@
         <v>39.44223107569721</v>
       </c>
       <c r="G45" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="H45" t="n">
         <v>47.60956175298804</v>
@@ -11912,7 +11936,7 @@
         <v>66.13545816733067</v>
       </c>
       <c r="G62" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="H62" t="n">
         <v>64.01062416998673</v>
@@ -12476,7 +12500,7 @@
         <v>62.15139442231076</v>
       </c>
       <c r="H79" t="n">
-        <v>50.33200531208499</v>
+        <v>50.332005312085</v>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
@@ -12608,7 +12632,7 @@
         <v>23.90438247011953</v>
       </c>
       <c r="H83" t="n">
-        <v>60.55776892430278</v>
+        <v>60.55776892430279</v>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
@@ -12740,7 +12764,7 @@
         <v>23.90438247011953</v>
       </c>
       <c r="H87" t="n">
-        <v>58.16733067729083</v>
+        <v>58.16733067729084</v>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
@@ -13532,7 +13556,7 @@
         <v>43.82470119521913</v>
       </c>
       <c r="H111" t="n">
-        <v>56.44090305444887</v>
+        <v>56.44090305444888</v>
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
@@ -13562,7 +13586,7 @@
         <v>50.59760956175299</v>
       </c>
       <c r="G112" t="n">
-        <v>3.585657370517922</v>
+        <v>3.585657370517921</v>
       </c>
       <c r="H112" t="n">
         <v>52.65604249667995</v>
@@ -13763,7 +13787,7 @@
         <v>12.35059760956176</v>
       </c>
       <c r="H118" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I118" s="3" t="inlineStr">
         <is>
@@ -13895,7 +13919,7 @@
         <v>64.9402390438247</v>
       </c>
       <c r="H122" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I122" s="3" t="inlineStr">
         <is>
@@ -14093,7 +14117,7 @@
         <v>43.82470119521913</v>
       </c>
       <c r="H128" t="n">
-        <v>52.25763612217795</v>
+        <v>52.25763612217796</v>
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
@@ -14387,7 +14411,7 @@
         <v>40.23904382470119</v>
       </c>
       <c r="G137" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="H137" t="n">
         <v>60.02656042496679</v>
@@ -14522,7 +14546,7 @@
         <v>5.179282868525888</v>
       </c>
       <c r="H141" t="n">
-        <v>53.91766268260291</v>
+        <v>53.91766268260292</v>
       </c>
       <c r="I141" s="3" t="inlineStr">
         <is>
@@ -14687,7 +14711,7 @@
         <v>97.60956175298804</v>
       </c>
       <c r="H146" t="n">
-        <v>50.13280212483399</v>
+        <v>50.132802124834</v>
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
@@ -14813,7 +14837,7 @@
         <v>22.70916334661354</v>
       </c>
       <c r="F150" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="G150" t="n">
         <v>74.10358565737052</v>
@@ -14867,7 +14891,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C152" t="n">
         <v>62.15139442231076</v>
@@ -14900,7 +14924,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>23.10756972111554</v>
+        <v>23.10756972111553</v>
       </c>
       <c r="C153" t="n">
         <v>44.22310756972112</v>
@@ -14951,7 +14975,7 @@
         <v>78.48605577689243</v>
       </c>
       <c r="H154" t="n">
-        <v>23.17397078353254</v>
+        <v>23.17397078353253</v>
       </c>
       <c r="I154" s="6" t="inlineStr">
         <is>
@@ -14966,7 +14990,7 @@
         </is>
       </c>
       <c r="B155" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="C155" t="n">
         <v>40.63745019920319</v>
@@ -14999,7 +15023,7 @@
         </is>
       </c>
       <c r="B156" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="C156" t="n">
         <v>28.28685258964143</v>
@@ -15296,7 +15320,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C165" t="n">
         <v>61.35458167330678</v>
@@ -15473,7 +15497,7 @@
         <v>21.91235059760956</v>
       </c>
       <c r="F170" t="n">
-        <v>24.30278884462151</v>
+        <v>24.30278884462152</v>
       </c>
       <c r="G170" t="n">
         <v>97.60956175298804</v>
@@ -15674,7 +15698,7 @@
         <v>82.47011952191235</v>
       </c>
       <c r="G176" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="H176" t="n">
         <v>45.08632138114209</v>
@@ -16460,7 +16484,7 @@
         <v>13.14741035856574</v>
       </c>
       <c r="E200" t="n">
-        <v>36.25498007968127</v>
+        <v>36.25498007968128</v>
       </c>
       <c r="F200" t="n">
         <v>4.382470119521913</v>
@@ -16766,7 +16790,7 @@
         <v>39.44223107569721</v>
       </c>
       <c r="H209" t="n">
-        <v>50.33200531208499</v>
+        <v>50.332005312085</v>
       </c>
       <c r="I209" s="3" t="inlineStr">
         <is>
@@ -16784,7 +16808,7 @@
         <v>11.55378486055777</v>
       </c>
       <c r="C210" t="n">
-        <v>20.31872509960159</v>
+        <v>20.3187250996016</v>
       </c>
       <c r="D210" t="n">
         <v>43.02788844621514</v>
@@ -17294,7 +17318,7 @@
         <v>87.25099601593625</v>
       </c>
       <c r="H225" t="n">
-        <v>36.12217795484727</v>
+        <v>36.12217795484728</v>
       </c>
       <c r="I225" s="4" t="inlineStr">
         <is>
@@ -17450,7 +17474,7 @@
         <v>45.0199203187251</v>
       </c>
       <c r="E230" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="F230" t="n">
         <v>19.9203187250996</v>
@@ -18266,7 +18290,7 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>27.09163346613546</v>
+        <v>27.09163346613545</v>
       </c>
       <c r="C255" t="n">
         <v>31.87250996015936</v>
@@ -18995,7 +19019,7 @@
         <v>31.87250996015936</v>
       </c>
       <c r="C277" t="n">
-        <v>29.88047808764939</v>
+        <v>29.8804780876494</v>
       </c>
       <c r="D277" t="n">
         <v>17.52988047808765</v>
@@ -19166,7 +19190,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>92.03187250996017</v>
+        <v>94.42231075697212</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -19175,7 +19199,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.32005312084993</v>
+        <v>53.71845949535192</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -19199,7 +19223,7 @@
         <v>42.62948207171315</v>
       </c>
       <c r="E283" t="n">
-        <v>98.80478087649402</v>
+        <v>100</v>
       </c>
       <c r="F283" t="n">
         <v>81.67330677290838</v>
@@ -19208,9 +19232,42 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H283" t="n">
-        <v>60.55776892430278</v>
+        <v>60.75697211155379</v>
       </c>
       <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>68.12749003984064</v>
+      </c>
+      <c r="C284" t="n">
+        <v>52.98804780876494</v>
+      </c>
+      <c r="D284" t="n">
+        <v>35.85657370517929</v>
+      </c>
+      <c r="E284" t="n">
+        <v>90.0398406374502</v>
+      </c>
+      <c r="F284" t="n">
+        <v>78.88446215139442</v>
+      </c>
+      <c r="G284" t="n">
+        <v>44.62151394422311</v>
+      </c>
+      <c r="H284" t="n">
+        <v>61.75298804780877</v>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
         <is>
           <t>Greed</t>
         </is>
@@ -19254,7 +19311,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-04 12:54 UTC</t>
+          <t>2026-08-04 14:57 UTC</t>
         </is>
       </c>
     </row>
@@ -19266,7 +19323,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>282 days, 2025-06-11 to 2026-08-03</t>
+          <t>283 days, 2025-06-11 to 2026-08-04</t>
         </is>
       </c>
     </row>
@@ -19278,7 +19335,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>282 days, 2025-06-11 to 2026-08-03</t>
+          <t>283 days, 2025-06-11 to 2026-08-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-08-05
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I284"/>
+  <dimension ref="A1:I285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9779,7 +9779,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>94.42231075697212</v>
+        <v>92.03187250996017</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -9788,7 +9788,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.71845949535192</v>
+        <v>53.32005312084993</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -9812,7 +9812,7 @@
         <v>42.62948207171315</v>
       </c>
       <c r="E283" t="n">
-        <v>100</v>
+        <v>98.80478087649402</v>
       </c>
       <c r="F283" t="n">
         <v>81.67330677290838</v>
@@ -9821,7 +9821,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H283" t="n">
-        <v>60.75697211155379</v>
+        <v>60.55776892430279</v>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
@@ -9842,10 +9842,10 @@
         <v>52.98804780876494</v>
       </c>
       <c r="D284" t="n">
-        <v>35.85657370517929</v>
+        <v>16.73306772908366</v>
       </c>
       <c r="E284" t="n">
-        <v>90.0398406374502</v>
+        <v>81.27490039840637</v>
       </c>
       <c r="F284" t="n">
         <v>78.88446215139442</v>
@@ -9854,9 +9854,42 @@
         <v>44.62151394422311</v>
       </c>
       <c r="H284" t="n">
-        <v>61.75298804780877</v>
+        <v>57.10491367861886</v>
       </c>
       <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>68.92430278884463</v>
+      </c>
+      <c r="C285" t="n">
+        <v>57.76892430278885</v>
+      </c>
+      <c r="D285" t="n">
+        <v>42.23107569721115</v>
+      </c>
+      <c r="E285" t="n">
+        <v>75.29880478087649</v>
+      </c>
+      <c r="F285" t="n">
+        <v>90.0398406374502</v>
+      </c>
+      <c r="G285" t="n">
+        <v>64.9402390438247</v>
+      </c>
+      <c r="H285" t="n">
+        <v>66.53386454183267</v>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
         <is>
           <t>Greed</t>
         </is>
@@ -9873,7 +9906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I284"/>
+  <dimension ref="A1:I285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19190,7 +19223,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>94.42231075697212</v>
+        <v>92.03187250996017</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -19199,7 +19232,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.71845949535192</v>
+        <v>53.32005312084993</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -19223,7 +19256,7 @@
         <v>42.62948207171315</v>
       </c>
       <c r="E283" t="n">
-        <v>100</v>
+        <v>98.80478087649402</v>
       </c>
       <c r="F283" t="n">
         <v>81.67330677290838</v>
@@ -19232,7 +19265,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H283" t="n">
-        <v>60.75697211155379</v>
+        <v>60.55776892430279</v>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
@@ -19253,10 +19286,10 @@
         <v>52.98804780876494</v>
       </c>
       <c r="D284" t="n">
-        <v>35.85657370517929</v>
+        <v>16.73306772908366</v>
       </c>
       <c r="E284" t="n">
-        <v>90.0398406374502</v>
+        <v>81.27490039840637</v>
       </c>
       <c r="F284" t="n">
         <v>78.88446215139442</v>
@@ -19265,9 +19298,42 @@
         <v>44.62151394422311</v>
       </c>
       <c r="H284" t="n">
-        <v>61.75298804780877</v>
+        <v>57.10491367861886</v>
       </c>
       <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>Greed</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>68.92430278884463</v>
+      </c>
+      <c r="C285" t="n">
+        <v>57.76892430278885</v>
+      </c>
+      <c r="D285" t="n">
+        <v>42.23107569721115</v>
+      </c>
+      <c r="E285" t="n">
+        <v>75.29880478087649</v>
+      </c>
+      <c r="F285" t="n">
+        <v>90.0398406374502</v>
+      </c>
+      <c r="G285" t="n">
+        <v>64.9402390438247</v>
+      </c>
+      <c r="H285" t="n">
+        <v>66.53386454183267</v>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
         <is>
           <t>Greed</t>
         </is>
@@ -19311,7 +19377,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-04 14:57 UTC</t>
+          <t>2026-08-05 14:43 UTC</t>
         </is>
       </c>
     </row>
@@ -19323,7 +19389,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>283 days, 2025-06-11 to 2026-08-04</t>
+          <t>284 days, 2025-06-11 to 2026-08-05</t>
         </is>
       </c>
     </row>
@@ -19335,7 +19401,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>283 days, 2025-06-11 to 2026-08-04</t>
+          <t>284 days, 2025-06-11 to 2026-08-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update India FGI — 2026-08-06
</commit_message>
<xml_diff>
--- a/docs/data/India_FearGreed_History.xlsx
+++ b/docs/data/India_FearGreed_History.xlsx
@@ -9779,7 +9779,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>92.03187250996017</v>
+        <v>94.42231075697212</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -9788,7 +9788,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.32005312084993</v>
+        <v>53.71845949535192</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -9812,7 +9812,7 @@
         <v>42.62948207171315</v>
       </c>
       <c r="E283" t="n">
-        <v>98.80478087649402</v>
+        <v>100</v>
       </c>
       <c r="F283" t="n">
         <v>81.67330677290838</v>
@@ -9821,7 +9821,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H283" t="n">
-        <v>60.55776892430279</v>
+        <v>60.75697211155379</v>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
@@ -9845,7 +9845,7 @@
         <v>16.73306772908366</v>
       </c>
       <c r="E284" t="n">
-        <v>81.27490039840637</v>
+        <v>89.24302788844621</v>
       </c>
       <c r="F284" t="n">
         <v>78.88446215139442</v>
@@ -9854,7 +9854,7 @@
         <v>44.62151394422311</v>
       </c>
       <c r="H284" t="n">
-        <v>57.10491367861886</v>
+        <v>58.43293492695884</v>
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
@@ -9878,7 +9878,7 @@
         <v>42.23107569721115</v>
       </c>
       <c r="E285" t="n">
-        <v>75.29880478087649</v>
+        <v>84.06374501992032</v>
       </c>
       <c r="F285" t="n">
         <v>90.0398406374502</v>
@@ -9887,7 +9887,7 @@
         <v>64.9402390438247</v>
       </c>
       <c r="H285" t="n">
-        <v>66.53386454183267</v>
+        <v>67.99468791500664</v>
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
@@ -19223,7 +19223,7 @@
         <v>43.02788844621514</v>
       </c>
       <c r="E282" t="n">
-        <v>92.03187250996017</v>
+        <v>94.42231075697212</v>
       </c>
       <c r="F282" t="n">
         <v>64.14342629482071</v>
@@ -19232,7 +19232,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H282" t="n">
-        <v>53.32005312084993</v>
+        <v>53.71845949535192</v>
       </c>
       <c r="I282" s="3" t="inlineStr">
         <is>
@@ -19256,7 +19256,7 @@
         <v>42.62948207171315</v>
       </c>
       <c r="E283" t="n">
-        <v>98.80478087649402</v>
+        <v>100</v>
       </c>
       <c r="F283" t="n">
         <v>81.67330677290838</v>
@@ -19265,7 +19265,7 @@
         <v>2.788844621513945</v>
       </c>
       <c r="H283" t="n">
-        <v>60.55776892430279</v>
+        <v>60.75697211155379</v>
       </c>
       <c r="I283" s="2" t="inlineStr">
         <is>
@@ -19289,7 +19289,7 @@
         <v>16.73306772908366</v>
       </c>
       <c r="E284" t="n">
-        <v>81.27490039840637</v>
+        <v>89.24302788844621</v>
       </c>
       <c r="F284" t="n">
         <v>78.88446215139442</v>
@@ -19298,7 +19298,7 @@
         <v>44.62151394422311</v>
       </c>
       <c r="H284" t="n">
-        <v>57.10491367861886</v>
+        <v>58.43293492695884</v>
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
@@ -19322,7 +19322,7 @@
         <v>42.23107569721115</v>
       </c>
       <c r="E285" t="n">
-        <v>75.29880478087649</v>
+        <v>84.06374501992032</v>
       </c>
       <c r="F285" t="n">
         <v>90.0398406374502</v>
@@ -19331,7 +19331,7 @@
         <v>64.9402390438247</v>
       </c>
       <c r="H285" t="n">
-        <v>66.53386454183267</v>
+        <v>67.99468791500664</v>
       </c>
       <c r="I285" s="2" t="inlineStr">
         <is>
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-05 14:43 UTC</t>
+          <t>2026-08-06 12:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>